<commit_message>
Respaldo estable antes de auditoría global responsiva
</commit_message>
<xml_diff>
--- a/public/templates/prog_conductores.xlsx
+++ b/public/templates/prog_conductores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\_CODE\app-territorios\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F5F7BFE-90E0-4818-9C5C-0115755E2912}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B1EFB00-E5FD-4E22-A5CC-76E82E2A8BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{9E0D7C96-BD73-4F6E-ACB5-14B6DEBFF278}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="10">
   <si>
     <t>CONGREGACIÓN "NUEVE DE OCTUBRE" 14282</t>
   </si>
@@ -66,27 +66,6 @@
   </si>
   <si>
     <t>TERRITORIO</t>
-  </si>
-  <si>
-    <t>LUNES</t>
-  </si>
-  <si>
-    <t>MARTES</t>
-  </si>
-  <si>
-    <t>MIÉRCOLES</t>
-  </si>
-  <si>
-    <t>JUEVES</t>
-  </si>
-  <si>
-    <t>VIERNES</t>
-  </si>
-  <si>
-    <t>SÁBADO</t>
-  </si>
-  <si>
-    <t>DOMINGO</t>
   </si>
 </sst>
 </file>
@@ -1239,27 +1218,13 @@
       <c r="A4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
       <c r="I4" s="31" t="s">
         <v>3</v>
       </c>

</xml_diff>